<commit_message>
translation for nested start lists
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/start/NestedStartList.xlsx
+++ b/owlcms/src/main/resources/templates/start/NestedStartList.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/Misc/usaw-owlcms/local/templates/start/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\start\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0435B5C-546A-FC48-B64A-70188C66A689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A271D7-79CA-41B5-9392-785A5C1CFC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1460" yWindow="500" windowWidth="39500" windowHeight="25100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -556,48 +554,18 @@
     <t>${competition.competitionName}</t>
   </si>
   <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Session</t>
-  </si>
-  <si>
     <t>${agi.ageGroup.code}</t>
   </si>
   <si>
     <t>${session.name}</t>
   </si>
   <si>
-    <t>Age</t>
-  </si>
-  <si>
-    <t>Group</t>
-  </si>
-  <si>
-    <t>Cat</t>
-  </si>
-  <si>
-    <t>Lot</t>
-  </si>
-  <si>
     <t>${athlete.age}</t>
   </si>
   <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
     <t>${athlete.entryTotal}</t>
   </si>
   <si>
-    <t>Team</t>
-  </si>
-  <si>
-    <t>Comps</t>
-  </si>
-  <si>
     <t>${session.athletes.0.ageGroup.gender}</t>
   </si>
   <si>
@@ -605,9 +573,6 @@
   </si>
   <si>
     <t>${athlete.lotNumber}</t>
-  </si>
-  <si>
-    <t>Gndr</t>
   </si>
   <si>
     <t>${athlete.ageGroupCodesAsString}</t>
@@ -632,6 +597,39 @@
   </si>
   <si>
     <t>${athlete.fullName}</t>
+  </si>
+  <si>
+    <t>${t.get("Group")}</t>
+  </si>
+  <si>
+    <t>${t.get("Competition.competitionDate")}</t>
+  </si>
+  <si>
+    <t>${t.get("Gender")}</t>
+  </si>
+  <si>
+    <t>${t.get("AgeGoup")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.Category")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.Lot")}</t>
+  </si>
+  <si>
+    <t>${t.get("Age")}</t>
+  </si>
+  <si>
+    <t>${t.get("Name")}</t>
+  </si>
+  <si>
+    <t>${t.get("EntryTotal")}</t>
+  </si>
+  <si>
+    <t>${t.get("Team")}</t>
+  </si>
+  <si>
+    <t>${t.get("Competitions")}</t>
   </si>
 </sst>
 </file>
@@ -717,7 +715,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -739,9 +737,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
@@ -1090,34 +1085,34 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="4.83203125" customWidth="1"/>
-    <col min="4" max="4" width="6.83203125" customWidth="1"/>
-    <col min="5" max="5" width="4.83203125" customWidth="1"/>
-    <col min="6" max="7" width="5.83203125" customWidth="1"/>
-    <col min="8" max="8" width="28.83203125" customWidth="1"/>
-    <col min="9" max="9" width="5.83203125" customWidth="1"/>
-    <col min="10" max="10" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" customWidth="1"/>
+    <col min="3" max="3" width="7.140625" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" customWidth="1"/>
+    <col min="5" max="5" width="4.85546875" customWidth="1"/>
+    <col min="6" max="7" width="5.85546875" customWidth="1"/>
+    <col min="8" max="8" width="28.85546875" customWidth="1"/>
+    <col min="9" max="9" width="5.85546875" customWidth="1"/>
+    <col min="10" max="10" width="28.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1125,77 +1120,77 @@
       <c r="E2" s="1"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="7" t="s">
+      <c r="E4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="F4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="G4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4" s="4" t="s">
         <v>8</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="K3" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>